<commit_message>
working 3D nodal stranded coils tests
</commit_message>
<xml_diff>
--- a/tests/coil_3D_ave/input_template.xlsx
+++ b/tests/coil_3D_ave/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -1386,7 +1386,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="21.14785714285714" customWidth="1" bestFit="1"/>
@@ -1413,7 +1413,7 @@
     <col min="22" max="22" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1479,6 +1479,74 @@
       </c>
       <c r="V1" s="1" t="s">
         <v>77</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1">
+        <v>0</v>
+      </c>
+      <c r="S2" s="1">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1">
+        <v>0</v>
+      </c>
+      <c r="U2" s="1">
+        <v>0</v>
+      </c>
+      <c r="V2" s="1">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>